<commit_message>
Redesign the interface and add canvas objects
Replace the Excel-style ribbon with a Mac toolbar and a Format/Organize
inspector, move sheet tabs above the grid, and restyle the grid in
Figures green. Charts become live canvas objects alongside text boxes,
shapes and pictures that can be moved, resized and layered, and are
saved in a Figures worksheet extension. Add Share, a highlighting rules
list, border line styles and an offscreen snapshot tool.

Release 2.0.0.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H7hh9k43kX2H8w3kFr1cSC
</commit_message>
<xml_diff>
--- a/Samples/Figures Templates.xlsx
+++ b/Samples/Figures Templates.xlsx
@@ -29,7 +29,7 @@
     <font>
       <b/>
       <sz val="20"/>
-      <color rgb="FF44546A"/>
+      <color rgb="FF1F3A2C"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -57,12 +57,12 @@
     <font>
       <i/>
       <sz val="11"/>
-      <color rgb="FF44546A"/>
+      <color rgb="FF1F3A2C"/>
       <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF44546A"/>
+      <color rgb="FF1F3A2C"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -75,13 +75,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF4472C4"/>
+        <fgColor rgb="FF1E9A57"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F6FC"/>
+        <fgColor rgb="FFF1F8F4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -99,7 +99,7 @@
       <right/>
       <top/>
       <bottom style="thin">
-        <color rgb="FFD9E1F2"/>
+        <color rgb="FFD5EBDD"/>
       </bottom>
       <diagonal/>
     </border>
@@ -107,10 +107,10 @@
       <left/>
       <right/>
       <top style="thin">
-        <color rgb="FF4472C4"/>
+        <color rgb="FF1E9A57"/>
       </top>
       <bottom style="double">
-        <color rgb="FF4472C4"/>
+        <color rgb="FF1E9A57"/>
       </bottom>
       <diagonal/>
     </border>
@@ -425,7 +425,7 @@
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="FF638EC6"/>
+        <color rgb="FF4CC38A"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>

</xml_diff>